<commit_message>
create profil dosen sinta
</commit_message>
<xml_diff>
--- a/public/dosen_universitas_ngudi_waluyo.xlsx
+++ b/public/dosen_universitas_ngudi_waluyo.xlsx
@@ -1779,22 +1779,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANA PUJI ASTUTI</t>
+          <t>AGITYA RESTI ERWIYANI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6146672</t>
+          <t>6082202</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 12</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1805,44 +1805,44 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>115</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AGITYA RESTI ERWIYANI</t>
+          <t>ANA PUJI ASTUTI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6082202</t>
+          <t>6146672</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 12</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1853,22 +1853,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>471</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>170</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
         </is>
       </c>
     </row>
@@ -1923,22 +1923,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PUJI LESTARI</t>
+          <t>IKA NILAWATI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6093197</t>
+          <t>6785923</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 10</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1949,44 +1949,44 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>303</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>150</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>195</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IKA NILAWATI</t>
+          <t>HANI IRHAMDESSETYA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6785923</t>
+          <t>6813565</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1997,44 +1997,44 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>408</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>80</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6813565</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HANI IRHAMDESSETYA</t>
+          <t>PUJI LESTARI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6813565</t>
+          <t>6093197</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 0GS H-Index : 10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -2045,22 +2045,22 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>130</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6813565</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
         </is>
       </c>
     </row>
@@ -3123,22 +3123,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FIKTINA VIFRI ISMIRIYAM</t>
+          <t>ISFAIZAH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>6138998</t>
+          <t>6085376</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Kebidanan (S1)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -3149,44 +3149,44 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>510</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISFAIZAH</t>
+          <t>FIKTINA VIFRI ISMIRIYAM</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>6085376</t>
+          <t>6138998</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Kebidanan (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 5</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -3197,22 +3197,22 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>391</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>85</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>175</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
         </is>
       </c>
     </row>
@@ -3651,22 +3651,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>HERI SUGIARTO</t>
+          <t>RATIH LAILY NURJANAH</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>5985236</t>
+          <t>6199137</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Kesehatan Masyarakat (S1)</t>
+          <t>Sastra Inggris (S1)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -3677,44 +3677,44 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>459</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RATIH LAILY NURJANAH</t>
+          <t>HERI SUGIARTO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>6199137</t>
+          <t>5985236</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sastra Inggris (S1)</t>
+          <t>Kesehatan Masyarakat (S1)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 2GS H-Index : 5</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3725,22 +3725,22 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>372</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
         </is>
       </c>
     </row>
@@ -5667,17 +5667,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>AR-RAHIIM INNASH</t>
+          <t>ARDA RADITYA TANTRA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>6895455</t>
+          <t>6832181</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Akuntansi Perpajakan (D4)</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -5693,39 +5693,39 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>138</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5741,44 +5741,44 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>PUJI AFIATNA</t>
+          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>6198595</t>
+          <t>6828552</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Gizi (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -5789,44 +5789,44 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>198</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>120</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
+          <t>PUJI AFIATNA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>6828552</t>
+          <t>6198595</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Gizi (S1)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 2GS H-Index : 7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5837,22 +5837,22 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>194</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
         </is>
       </c>
     </row>
@@ -6099,22 +6099,22 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KARTIKA SARI</t>
+          <t>MUKHAMAD MUSTAIN</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>6080653</t>
+          <t>6668043</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Pendidikan Profesi Bidan (Profesi)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -6125,7 +6125,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>181</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6135,34 +6135,34 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6080653</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6668043</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MUKHAMAD MUSTAIN</t>
+          <t>KARTIKA SARI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>6668043</t>
+          <t>6080653</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Pendidikan Profesi Bidan (Profesi)</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -6173,7 +6173,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>155</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6183,12 +6183,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6668043</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6080653</t>
         </is>
       </c>
     </row>
@@ -6723,22 +6723,22 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SUWANTI</t>
+          <t>SALSABIELA DWIYUDRISA SUYUDI</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>6198864</t>
+          <t>6828726</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 2</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -6749,44 +6749,44 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>75</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198864</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828726</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SALSABIELA DWIYUDRISA SUYUDI</t>
+          <t>SUWANTI</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>6828726</t>
+          <t>6198864</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 2</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -6797,22 +6797,22 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>149</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828726</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198864</t>
         </is>
       </c>
     </row>
@@ -8163,17 +8163,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>DWI WISNU KURNIAWAN</t>
+          <t>FIKRI ARIYAD</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>6967441</t>
+          <t>6837372</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -8189,7 +8189,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -8204,29 +8204,29 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>FIKRI ARIYAD</t>
+          <t>MUFTI AGUNG WIBOWO</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>6837372</t>
+          <t>6871253</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Bisnis Digital (S1)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 1GS H-Index : 0</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -8237,44 +8237,44 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MUFTI AGUNG WIBOWO</t>
+          <t>DWI WISNU KURNIAWAN</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>6871253</t>
+          <t>6967441</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Bisnis Digital (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 1GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -8285,7 +8285,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -8295,12 +8295,12 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Styling halaman daftar riset dosen
</commit_message>
<xml_diff>
--- a/public/dosen_universitas_ngudi_waluyo.xlsx
+++ b/public/dosen_universitas_ngudi_waluyo.xlsx
@@ -1779,22 +1779,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANA PUJI ASTUTI</t>
+          <t>AGITYA RESTI ERWIYANI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6146672</t>
+          <t>6082202</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 12</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1805,44 +1805,44 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>115</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AGITYA RESTI ERWIYANI</t>
+          <t>ANA PUJI ASTUTI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6082202</t>
+          <t>6146672</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 12</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1853,22 +1853,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>471</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>170</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
         </is>
       </c>
     </row>
@@ -1971,22 +1971,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PUJI LESTARI</t>
+          <t>IKA NILAWATI</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6093197</t>
+          <t>6785923</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 10</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1997,44 +1997,44 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>303</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>150</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>195</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IKA NILAWATI</t>
+          <t>PUJI LESTARI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6785923</t>
+          <t>6093197</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -2045,22 +2045,22 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>130</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
         </is>
       </c>
     </row>
@@ -3171,22 +3171,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISFAIZAH</t>
+          <t>FIKTINA VIFRI ISMIRIYAM</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>6085376</t>
+          <t>6138998</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Kebidanan (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 5</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -3197,44 +3197,44 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>391</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>85</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>175</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FIKTINA VIFRI ISMIRIYAM</t>
+          <t>ISFAIZAH</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>6138998</t>
+          <t>6085376</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Kebidanan (S1)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -3245,22 +3245,22 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>510</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
         </is>
       </c>
     </row>
@@ -3699,22 +3699,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>HERI SUGIARTO</t>
+          <t>RATIH LAILY NURJANAH</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>5985236</t>
+          <t>6199137</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Kesehatan Masyarakat (S1)</t>
+          <t>Sastra Inggris (S1)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3725,44 +3725,44 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>459</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RATIH LAILY NURJANAH</t>
+          <t>HERI SUGIARTO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>6199137</t>
+          <t>5985236</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Sastra Inggris (S1)</t>
+          <t>Kesehatan Masyarakat (S1)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 2GS H-Index : 5</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3773,22 +3773,22 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>372</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
         </is>
       </c>
     </row>
@@ -5763,17 +5763,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5789,44 +5789,44 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>PUJI AFIATNA</t>
+          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>6198595</t>
+          <t>6828552</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Gizi (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5837,44 +5837,44 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>198</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>120</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
+          <t>PUJI AFIATNA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>6828552</t>
+          <t>6198595</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Gizi (S1)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 2GS H-Index : 7</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -5885,22 +5885,22 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>194</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
         </is>
       </c>
     </row>
@@ -6147,22 +6147,22 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MUKHAMAD MUSTAIN</t>
+          <t>KARTIKA SARI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>6668043</t>
+          <t>6080653</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Pendidikan Profesi Bidan (Profesi)</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -6173,7 +6173,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>155</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6183,34 +6183,34 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6668043</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6080653</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KARTIKA SARI</t>
+          <t>MUKHAMAD MUSTAIN</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>6080653</t>
+          <t>6668043</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Pendidikan Profesi Bidan (Profesi)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>181</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -6231,12 +6231,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6080653</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6668043</t>
         </is>
       </c>
     </row>
@@ -6771,22 +6771,22 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SALSABIELA DWIYUDRISA SUYUDI</t>
+          <t>SUWANTI</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>6828726</t>
+          <t>6198864</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 2</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -6797,44 +6797,44 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>149</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828726</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198864</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SUWANTI</t>
+          <t>SALSABIELA DWIYUDRISA SUYUDI</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>6198864</t>
+          <t>6828726</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 2</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -6845,22 +6845,22 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>75</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198864</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828726</t>
         </is>
       </c>
     </row>
@@ -7923,22 +7923,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SUKARNO</t>
+          <t>TUSI WIRAHAYU PERTIWI</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>6198543</t>
+          <t>6967446</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 14</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7964,29 +7964,29 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TUSI WIRAHAYU PERTIWI</t>
+          <t>SUKARNO</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>6967446</t>
+          <t>6198543</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 14</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>356</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -8012,19 +8012,19 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>INDAH KURNIAWATI</t>
+          <t>SITI KHOIRIYAH</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6910777</t>
+          <t>6910724</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8060,29 +8060,29 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SITI KHOIRIYAH</t>
+          <t>FITRIA PRIMI ASTUTI</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>6910724</t>
+          <t>6082432</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>174</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -8108,29 +8108,29 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FITRIA PRIMI ASTUTI</t>
+          <t>ANDI PRADANA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>6082432</t>
+          <t>6910783</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 1</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -8141,7 +8141,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910783</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
set tambah data manual
</commit_message>
<xml_diff>
--- a/public/dosen_universitas_ngudi_waluyo.xlsx
+++ b/public/dosen_universitas_ngudi_waluyo.xlsx
@@ -3699,22 +3699,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>HERI SUGIARTO</t>
+          <t>RATIH LAILY NURJANAH</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>5985236</t>
+          <t>6199137</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Kesehatan Masyarakat (S1)</t>
+          <t>Sastra Inggris (S1)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3725,44 +3725,44 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>459</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RATIH LAILY NURJANAH</t>
+          <t>HERI SUGIARTO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>6199137</t>
+          <t>5985236</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Sastra Inggris (S1)</t>
+          <t>Kesehatan Masyarakat (S1)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 2GS H-Index : 5</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3773,22 +3773,22 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>372</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
         </is>
       </c>
     </row>
@@ -5715,17 +5715,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5741,39 +5741,39 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5789,44 +5789,44 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>PUJI AFIATNA</t>
+          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>6198595</t>
+          <t>6828552</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Gizi (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5837,44 +5837,44 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>198</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>120</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
+          <t>PUJI AFIATNA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>6828552</t>
+          <t>6198595</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Gizi (S1)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 2GS H-Index : 7</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -5885,22 +5885,22 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>194</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
         </is>
       </c>
     </row>
@@ -7923,22 +7923,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SUKARNO</t>
+          <t>TUSI WIRAHAYU PERTIWI</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>6198543</t>
+          <t>6967446</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 14</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7964,29 +7964,29 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TUSI WIRAHAYU PERTIWI</t>
+          <t>SUKARNO</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>6967446</t>
+          <t>6198543</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 14</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>356</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -8012,19 +8012,19 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>INDAH KURNIAWATI</t>
+          <t>SITI KHOIRIYAH</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6910777</t>
+          <t>6910724</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8060,29 +8060,29 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SITI KHOIRIYAH</t>
+          <t>FITRIA PRIMI ASTUTI</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>6910724</t>
+          <t>6082432</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>174</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -8108,29 +8108,29 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FITRIA PRIMI ASTUTI</t>
+          <t>ANDI PRADANA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>6082432</t>
+          <t>6910783</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 1</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -8141,7 +8141,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -8156,19 +8156,19 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910783</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SITI KHOIRIYAH</t>
+          <t>ANDI PRADANA</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>6910724</t>
+          <t>6910783</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 1</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -8189,7 +8189,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -8204,24 +8204,24 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910783</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DWI WISNU KURNIAWAN</t>
+          <t>FIKRI ARIYAD</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>6967441</t>
+          <t>6837372</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -8237,7 +8237,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -8252,29 +8252,29 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>FIKRI ARIYAD</t>
+          <t>MUFTI AGUNG WIBOWO</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>6837372</t>
+          <t>6871253</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Bisnis Digital (S1)</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 1GS H-Index : 0</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -8285,44 +8285,44 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MUFTI AGUNG WIBOWO</t>
+          <t>DWI RETNA SUSILOWATI</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>6871253</t>
+          <t>6895451</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Bisnis Digital (S1)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 1GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -8333,7 +8333,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -8343,29 +8343,29 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>DWI RETNA SUSILOWATI</t>
+          <t>ADI PURWANTO</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>6895451</t>
+          <t>6198866</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -8381,39 +8381,39 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr">
+      <c r="I166" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ADI PURWANTO</t>
+          <t>DWI WISNU KURNIAWAN</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>6198866</t>
+          <t>6967441</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
         </is>
       </c>
     </row>

</xml_diff>